<commit_message>
refactor(lint+types): fix ruff lint violations and mypy errors
Resolve all ruff check and mypy issues introduced with strict tooling:

- commands/stocks/__init__.py: replace wildcard import with explicit
  imports; fix _get_hint/_get_code isinstance guards; annotate
  getPerformanceIdBySymbol return type as str
- commands/stocks/SpreedSheetComparation.py: replace wildcard import
  with explicit; annotate workbook as Workbook | None; add assert guard
- commands/stocks/morning_star.py: session.headers.update() instead of
  direct assignment (TypedDict compat); use getenv() or '' fallback
- commands/utils/tables.py: replace Union[...] with PEP 604 X | Y syntax
- stockstory/adapter_repo.py: add Any annotations for periods/series/out
- stockstory/collect.py: remove sys.exit(main()) since main() returns None
</commit_message>
<xml_diff>
--- a/assets/base-sheet.xlsx
+++ b/assets/base-sheet.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
   <si>
     <t xml:space="preserve">RATIOS</t>
   </si>
@@ -99,19 +99,20 @@
   <si>
     <t xml:space="preserve">VF/P %</t>
   </si>
+  <si>
+    <t xml:space="preserve">avg-valuation date</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="General"/>
-    <numFmt numFmtId="166" formatCode="[RED]0.00%;[BLUE]\-0.00%"/>
-    <numFmt numFmtId="167" formatCode="#,##0.00"/>
-    <numFmt numFmtId="168" formatCode="0.00%"/>
+    <numFmt numFmtId="165" formatCode="[RED]0.00%;[BLUE]\-0.00%"/>
+    <numFmt numFmtId="166" formatCode="0.00%"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -181,7 +182,6 @@
     </font>
     <font>
       <sz val="14"/>
-      <color rgb="FF000000"/>
       <name val="Work sans"/>
       <family val="0"/>
       <charset val="1"/>
@@ -189,6 +189,13 @@
     <font>
       <sz val="14"/>
       <color rgb="FF434343"/>
+      <name val="Work sans"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
       <name val="Work sans"/>
       <family val="0"/>
       <charset val="1"/>
@@ -205,6 +212,12 @@
       <sz val="14"/>
       <color rgb="FF073763"/>
       <name val="Work sans"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -478,7 +491,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="41">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -523,19 +536,107 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="11" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="3" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -543,119 +644,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="11" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="5" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="5" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="5" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="5" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="5" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="5" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="5" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="3" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="5" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="5" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -663,11 +652,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -751,37 +736,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -855,7 +840,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:T1009"/>
-  <sheetFormatPr defaultColWidth="8.6171875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6171875" defaultRowHeight="13.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="0.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26.88"/>
@@ -921,7 +906,7 @@
       <c r="D3" s="10"/>
       <c r="E3" s="10"/>
       <c r="F3" s="11" t="e">
-        <f aca="false">AVERAGE(C3,D3,E3)</f>
+        <f aca="false">AVERAGE(C3:E3)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="G3" s="8"/>
@@ -944,7 +929,7 @@
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
       <c r="F4" s="11" t="e">
-        <f aca="false">AVERAGE(C4,D4,E4)</f>
+        <f aca="false">AVERAGE(C4:E4)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="G4" s="8"/>
@@ -967,7 +952,7 @@
       <c r="D5" s="10"/>
       <c r="E5" s="10"/>
       <c r="F5" s="11" t="e">
-        <f aca="false">AVERAGE(C5,D5,E5)</f>
+        <f aca="false">AVERAGE(C5:E5)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="G5" s="8"/>
@@ -990,7 +975,7 @@
       <c r="D6" s="10"/>
       <c r="E6" s="10"/>
       <c r="F6" s="11" t="e">
-        <f aca="false">AVERAGE(C6,D6,E6)</f>
+        <f aca="false">AVERAGE(C6:E6)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="G6" s="8"/>
@@ -1013,7 +998,7 @@
       <c r="D7" s="10"/>
       <c r="E7" s="10"/>
       <c r="F7" s="11" t="e">
-        <f aca="false">AVERAGE(C7,D7,E7)</f>
+        <f aca="false">AVERAGE(C7:E7)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="G7" s="8"/>
@@ -1044,8 +1029,8 @@
         <f aca="false">365/E7</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="F8" s="14" t="e">
-        <f aca="false">AVERAGE(C8,D8,E8)</f>
+      <c r="F8" s="11" t="e">
+        <f aca="false">AVERAGE(C8:E8)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="G8" s="8"/>
@@ -1067,15 +1052,15 @@
       <c r="C9" s="13"/>
       <c r="D9" s="13"/>
       <c r="E9" s="13"/>
-      <c r="F9" s="14" t="e">
-        <f aca="false">AVERAGE(C9,D9,E9)</f>
+      <c r="F9" s="11" t="e">
+        <f aca="false">AVERAGE(C9:E9)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="G9" s="8"/>
       <c r="H9" s="8"/>
-      <c r="I9" s="15"/>
-      <c r="J9" s="15"/>
-      <c r="K9" s="15"/>
+      <c r="I9" s="14"/>
+      <c r="J9" s="14"/>
+      <c r="K9" s="14"/>
       <c r="L9" s="4"/>
       <c r="M9" s="4"/>
       <c r="N9" s="4"/>
@@ -1091,18 +1076,18 @@
       <c r="B10" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="16"/>
-      <c r="D10" s="16"/>
-      <c r="E10" s="16"/>
-      <c r="F10" s="17" t="e">
-        <f aca="false">AVERAGE(C10,D10,E10)</f>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="11" t="e">
+        <f aca="false">AVERAGE(C10:E10)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="G10" s="8"/>
       <c r="H10" s="8"/>
-      <c r="I10" s="15"/>
-      <c r="J10" s="15"/>
-      <c r="K10" s="15"/>
+      <c r="I10" s="14"/>
+      <c r="J10" s="14"/>
+      <c r="K10" s="14"/>
       <c r="L10" s="4"/>
       <c r="M10" s="4"/>
       <c r="N10" s="4"/>
@@ -1118,18 +1103,18 @@
       <c r="B11" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="16"/>
-      <c r="D11" s="16"/>
-      <c r="E11" s="16"/>
-      <c r="F11" s="17" t="e">
-        <f aca="false">AVERAGE(C11,D11,E11)</f>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="11" t="e">
+        <f aca="false">AVERAGE(C11:E11)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="G11" s="8"/>
       <c r="H11" s="8"/>
-      <c r="I11" s="15"/>
-      <c r="J11" s="15"/>
-      <c r="K11" s="15"/>
+      <c r="I11" s="14"/>
+      <c r="J11" s="14"/>
+      <c r="K11" s="14"/>
       <c r="L11" s="4"/>
       <c r="M11" s="4"/>
       <c r="N11" s="4"/>
@@ -1149,14 +1134,14 @@
       <c r="D12" s="10"/>
       <c r="E12" s="10"/>
       <c r="F12" s="11" t="e">
-        <f aca="false">AVERAGE(C12,D12,E12)</f>
+        <f aca="false">AVERAGE(C12:E12)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="G12" s="8"/>
       <c r="H12" s="8"/>
-      <c r="I12" s="15"/>
-      <c r="J12" s="15"/>
-      <c r="K12" s="15"/>
+      <c r="I12" s="14"/>
+      <c r="J12" s="14"/>
+      <c r="K12" s="14"/>
       <c r="L12" s="4"/>
       <c r="M12" s="4"/>
       <c r="N12" s="4"/>
@@ -1176,14 +1161,14 @@
       <c r="D13" s="10"/>
       <c r="E13" s="10"/>
       <c r="F13" s="11" t="e">
-        <f aca="false">AVERAGE(C13,D13,E13)</f>
+        <f aca="false">AVERAGE(C13:E13)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="G13" s="8"/>
       <c r="H13" s="8"/>
-      <c r="I13" s="15"/>
-      <c r="J13" s="15"/>
-      <c r="K13" s="15"/>
+      <c r="I13" s="14"/>
+      <c r="J13" s="14"/>
+      <c r="K13" s="14"/>
       <c r="L13" s="4"/>
       <c r="M13" s="4"/>
       <c r="N13" s="4"/>
@@ -1203,14 +1188,14 @@
       <c r="D14" s="10"/>
       <c r="E14" s="10"/>
       <c r="F14" s="11" t="e">
-        <f aca="false">AVERAGE(C14,D14,E14)</f>
+        <f aca="false">AVERAGE(C14:E14)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="G14" s="8"/>
       <c r="H14" s="8"/>
-      <c r="I14" s="15"/>
-      <c r="J14" s="15"/>
-      <c r="K14" s="15"/>
+      <c r="I14" s="14"/>
+      <c r="J14" s="14"/>
+      <c r="K14" s="14"/>
       <c r="L14" s="4"/>
       <c r="M14" s="4"/>
       <c r="N14" s="4"/>
@@ -1223,21 +1208,21 @@
     </row>
     <row r="15" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4"/>
-      <c r="B15" s="18" t="s">
+      <c r="B15" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="20" t="e">
-        <f aca="false">AVERAGE(C15,D15,E15)</f>
+      <c r="C15" s="17"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="11" t="e">
+        <f aca="false">AVERAGE(C15:E15)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="G15" s="8"/>
       <c r="H15" s="8"/>
-      <c r="I15" s="15"/>
-      <c r="J15" s="15"/>
-      <c r="K15" s="15"/>
+      <c r="I15" s="14"/>
+      <c r="J15" s="14"/>
+      <c r="K15" s="14"/>
       <c r="L15" s="4"/>
       <c r="M15" s="4"/>
       <c r="N15" s="4"/>
@@ -1250,16 +1235,16 @@
     </row>
     <row r="16" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4"/>
-      <c r="B16" s="21"/>
+      <c r="B16" s="18"/>
       <c r="C16" s="8"/>
       <c r="D16" s="8"/>
       <c r="E16" s="8"/>
       <c r="F16" s="8"/>
       <c r="G16" s="8"/>
       <c r="H16" s="8"/>
-      <c r="I16" s="15"/>
-      <c r="J16" s="15"/>
-      <c r="K16" s="15"/>
+      <c r="I16" s="14"/>
+      <c r="J16" s="14"/>
+      <c r="K16" s="14"/>
       <c r="L16" s="4"/>
       <c r="M16" s="4"/>
       <c r="N16" s="4"/>
@@ -1289,9 +1274,9 @@
       </c>
       <c r="G17" s="8"/>
       <c r="H17" s="8"/>
-      <c r="I17" s="15"/>
-      <c r="J17" s="15"/>
-      <c r="K17" s="15"/>
+      <c r="I17" s="14"/>
+      <c r="J17" s="14"/>
+      <c r="K17" s="14"/>
       <c r="L17" s="4"/>
       <c r="M17" s="4"/>
       <c r="N17" s="4"/>
@@ -1307,14 +1292,14 @@
       <c r="B18" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C18" s="22"/>
-      <c r="D18" s="22"/>
-      <c r="E18" s="23"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="19"/>
       <c r="G18" s="8"/>
       <c r="H18" s="8"/>
-      <c r="I18" s="15"/>
-      <c r="J18" s="15"/>
-      <c r="K18" s="15"/>
+      <c r="I18" s="14"/>
+      <c r="J18" s="14"/>
+      <c r="K18" s="14"/>
       <c r="L18" s="4"/>
       <c r="M18" s="4"/>
       <c r="N18" s="4"/>
@@ -1330,23 +1315,23 @@
       <c r="B19" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C19" s="24" t="e">
+      <c r="C19" s="20" t="e">
         <f aca="false">(C$18*$F12)/C12</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D19" s="25" t="e">
+      <c r="D19" s="21" t="e">
         <f aca="false">(D$18*$F12)/D12</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E19" s="26" t="e">
+      <c r="E19" s="19" t="e">
         <f aca="false">(E$18*$F12)/E12</f>
         <v>#DIV/0!</v>
       </c>
       <c r="G19" s="8"/>
       <c r="H19" s="8"/>
-      <c r="I19" s="15"/>
-      <c r="J19" s="15"/>
-      <c r="K19" s="15"/>
+      <c r="I19" s="14"/>
+      <c r="J19" s="14"/>
+      <c r="K19" s="14"/>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
       <c r="N19" s="4"/>
@@ -1362,23 +1347,23 @@
       <c r="B20" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C20" s="27" t="e">
+      <c r="C20" s="22" t="e">
         <f aca="false">(C$18*$F13)/C13</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D20" s="26" t="e">
+      <c r="D20" s="19" t="e">
         <f aca="false">(D$18*$F13)/D13</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E20" s="26" t="e">
+      <c r="E20" s="19" t="e">
         <f aca="false">(E$18*$F13)/E13</f>
         <v>#DIV/0!</v>
       </c>
       <c r="G20" s="8"/>
       <c r="H20" s="8"/>
-      <c r="I20" s="15"/>
-      <c r="J20" s="15"/>
-      <c r="K20" s="15"/>
+      <c r="I20" s="14"/>
+      <c r="J20" s="14"/>
+      <c r="K20" s="14"/>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
       <c r="N20" s="4"/>
@@ -1394,23 +1379,23 @@
       <c r="B21" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="C21" s="27" t="e">
+      <c r="C21" s="22" t="e">
         <f aca="false">(C$18*$F14)/C14</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D21" s="26" t="e">
+      <c r="D21" s="19" t="e">
         <f aca="false">(D$18*$F14)/D14</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E21" s="26" t="e">
+      <c r="E21" s="19" t="e">
         <f aca="false">(E$18*$F14)/E14</f>
         <v>#DIV/0!</v>
       </c>
       <c r="G21" s="8"/>
       <c r="H21" s="8"/>
-      <c r="I21" s="15"/>
-      <c r="J21" s="15"/>
-      <c r="K21" s="15"/>
+      <c r="I21" s="14"/>
+      <c r="J21" s="14"/>
+      <c r="K21" s="14"/>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
       <c r="N21" s="4"/>
@@ -1423,26 +1408,26 @@
     </row>
     <row r="22" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4"/>
-      <c r="B22" s="18" t="s">
+      <c r="B22" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="C22" s="28" t="e">
+      <c r="C22" s="23" t="e">
         <f aca="false">(C$18*$F15)/C15</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D22" s="29" t="e">
+      <c r="D22" s="24" t="e">
         <f aca="false">(D$18*$F15)/D15</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E22" s="29" t="e">
+      <c r="E22" s="24" t="e">
         <f aca="false">(E$18*$F15)/E15</f>
         <v>#DIV/0!</v>
       </c>
       <c r="G22" s="8"/>
       <c r="H22" s="8"/>
-      <c r="I22" s="15"/>
-      <c r="J22" s="15"/>
-      <c r="K22" s="15"/>
+      <c r="I22" s="14"/>
+      <c r="J22" s="14"/>
+      <c r="K22" s="14"/>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
       <c r="N22" s="4"/>
@@ -1462,9 +1447,9 @@
       <c r="F23" s="8"/>
       <c r="G23" s="8"/>
       <c r="H23" s="8"/>
-      <c r="I23" s="15"/>
-      <c r="J23" s="15"/>
-      <c r="K23" s="15"/>
+      <c r="I23" s="14"/>
+      <c r="J23" s="14"/>
+      <c r="K23" s="14"/>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
       <c r="N23" s="4"/>
@@ -1492,8 +1477,8 @@
         <f aca="false">E2</f>
         <v>0</v>
       </c>
-      <c r="G24" s="30"/>
-      <c r="H24" s="30"/>
+      <c r="G24" s="25"/>
+      <c r="H24" s="25"/>
       <c r="I24" s="4"/>
       <c r="J24" s="4"/>
       <c r="K24" s="4"/>
@@ -1513,20 +1498,20 @@
         <f aca="false">B12</f>
         <v>PER</v>
       </c>
-      <c r="C25" s="22" t="n">
+      <c r="C25" s="10" t="n">
         <f aca="false">C12</f>
         <v>0</v>
       </c>
-      <c r="D25" s="22" t="n">
+      <c r="D25" s="10" t="n">
         <f aca="false">D12</f>
         <v>0</v>
       </c>
-      <c r="E25" s="22" t="n">
+      <c r="E25" s="10" t="n">
         <f aca="false">E12</f>
         <v>0</v>
       </c>
-      <c r="G25" s="30"/>
-      <c r="H25" s="30"/>
+      <c r="G25" s="25"/>
+      <c r="H25" s="25"/>
       <c r="I25" s="4"/>
       <c r="J25" s="4"/>
       <c r="K25" s="4"/>
@@ -1546,11 +1531,11 @@
         <f aca="false">B25 &amp; " 5-Yr"</f>
         <v>PER 5-Yr</v>
       </c>
-      <c r="C26" s="22"/>
-      <c r="D26" s="31"/>
-      <c r="E26" s="11"/>
-      <c r="G26" s="30"/>
-      <c r="H26" s="30"/>
+      <c r="C26" s="10"/>
+      <c r="D26" s="10"/>
+      <c r="E26" s="10"/>
+      <c r="G26" s="25"/>
+      <c r="H26" s="25"/>
       <c r="I26" s="4"/>
       <c r="J26" s="4"/>
       <c r="K26" s="4"/>
@@ -1566,24 +1551,24 @@
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="4"/>
-      <c r="B27" s="32" t="str">
+      <c r="B27" s="26" t="str">
         <f aca="false">"Valuacion " &amp; B26</f>
         <v>Valuacion PER 5-Yr</v>
       </c>
-      <c r="C27" s="33" t="e">
+      <c r="C27" s="27" t="e">
         <f aca="false">(C$18*C26)/C25</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D27" s="33" t="e">
+      <c r="D27" s="27" t="e">
         <f aca="false">(D$18*D26)/D25</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E27" s="34" t="e">
+      <c r="E27" s="28" t="e">
         <f aca="false">(E$18*E26)/E25</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="G27" s="30"/>
-      <c r="H27" s="30"/>
+      <c r="G27" s="25"/>
+      <c r="H27" s="25"/>
       <c r="I27" s="4"/>
       <c r="J27" s="4"/>
       <c r="K27" s="4"/>
@@ -1603,20 +1588,20 @@
         <f aca="false">B13</f>
         <v>PCF</v>
       </c>
-      <c r="C28" s="33" t="n">
+      <c r="C28" s="27" t="n">
         <f aca="false">C13</f>
         <v>0</v>
       </c>
-      <c r="D28" s="33" t="n">
+      <c r="D28" s="27" t="n">
         <f aca="false">D13</f>
         <v>0</v>
       </c>
-      <c r="E28" s="33" t="n">
+      <c r="E28" s="27" t="n">
         <f aca="false">E13</f>
         <v>0</v>
       </c>
-      <c r="G28" s="30"/>
-      <c r="H28" s="30"/>
+      <c r="G28" s="25"/>
+      <c r="H28" s="25"/>
       <c r="I28" s="4"/>
       <c r="J28" s="4"/>
       <c r="K28" s="4"/>
@@ -1636,11 +1621,11 @@
         <f aca="false">B28 &amp; " 5-Yr"</f>
         <v>PCF 5-Yr</v>
       </c>
-      <c r="C29" s="33"/>
-      <c r="D29" s="33"/>
-      <c r="E29" s="34"/>
-      <c r="G29" s="30"/>
-      <c r="H29" s="30"/>
+      <c r="C29" s="27"/>
+      <c r="D29" s="27"/>
+      <c r="E29" s="28"/>
+      <c r="G29" s="25"/>
+      <c r="H29" s="25"/>
       <c r="I29" s="4"/>
       <c r="J29" s="4"/>
       <c r="K29" s="4"/>
@@ -1656,24 +1641,24 @@
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="4"/>
-      <c r="B30" s="32" t="str">
+      <c r="B30" s="26" t="str">
         <f aca="false">"Valuacion " &amp; B29</f>
         <v>Valuacion PCF 5-Yr</v>
       </c>
-      <c r="C30" s="33" t="e">
+      <c r="C30" s="27" t="e">
         <f aca="false">(C$18*C29)/C28</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D30" s="33" t="e">
+      <c r="D30" s="27" t="e">
         <f aca="false">(D$18*D29)/D28</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E30" s="33" t="e">
+      <c r="E30" s="27" t="e">
         <f aca="false">(E$18*E29)/E28</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="G30" s="30"/>
-      <c r="H30" s="30"/>
+      <c r="G30" s="25"/>
+      <c r="H30" s="25"/>
       <c r="I30" s="4"/>
       <c r="J30" s="4"/>
       <c r="K30" s="4"/>
@@ -1693,20 +1678,20 @@
         <f aca="false">B14</f>
         <v>PS</v>
       </c>
-      <c r="C31" s="31" t="n">
+      <c r="C31" s="10" t="n">
         <f aca="false">C14</f>
         <v>0</v>
       </c>
-      <c r="D31" s="31" t="n">
+      <c r="D31" s="10" t="n">
         <f aca="false">D14</f>
         <v>0</v>
       </c>
-      <c r="E31" s="31" t="n">
+      <c r="E31" s="10" t="n">
         <f aca="false">E14</f>
         <v>0</v>
       </c>
-      <c r="G31" s="30"/>
-      <c r="H31" s="30"/>
+      <c r="G31" s="25"/>
+      <c r="H31" s="25"/>
       <c r="I31" s="4"/>
       <c r="J31" s="4"/>
       <c r="K31" s="4"/>
@@ -1726,11 +1711,11 @@
         <f aca="false">B31 &amp; " 5-Yr"</f>
         <v>PS 5-Yr</v>
       </c>
-      <c r="C32" s="31"/>
-      <c r="D32" s="31"/>
-      <c r="E32" s="11"/>
-      <c r="G32" s="30"/>
-      <c r="H32" s="30"/>
+      <c r="C32" s="10"/>
+      <c r="D32" s="10"/>
+      <c r="E32" s="10"/>
+      <c r="G32" s="25"/>
+      <c r="H32" s="25"/>
       <c r="I32" s="4"/>
       <c r="J32" s="4"/>
       <c r="K32" s="4"/>
@@ -1746,24 +1731,24 @@
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="4"/>
-      <c r="B33" s="32" t="str">
+      <c r="B33" s="26" t="str">
         <f aca="false">"Valuacion " &amp; B32</f>
         <v>Valuacion PS 5-Yr</v>
       </c>
-      <c r="C33" s="35" t="e">
+      <c r="C33" s="27" t="e">
         <f aca="false">(C$18*C32)/C31</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D33" s="35" t="e">
+      <c r="D33" s="27" t="e">
         <f aca="false">(D$18*D32)/D31</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E33" s="36" t="e">
+      <c r="E33" s="28" t="e">
         <f aca="false">(E$18*E32)/E31</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="G33" s="30"/>
-      <c r="H33" s="30"/>
+      <c r="G33" s="25"/>
+      <c r="H33" s="25"/>
       <c r="I33" s="4"/>
       <c r="J33" s="4"/>
       <c r="K33" s="4"/>
@@ -1779,23 +1764,23 @@
     </row>
     <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="4"/>
-      <c r="B34" s="37" t="s">
+      <c r="B34" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="C34" s="38" t="n">
+      <c r="C34" s="30" t="n">
         <f aca="false">C15</f>
         <v>0</v>
       </c>
-      <c r="D34" s="38" t="n">
+      <c r="D34" s="30" t="n">
         <f aca="false">D15</f>
         <v>0</v>
       </c>
-      <c r="E34" s="38" t="n">
+      <c r="E34" s="30" t="n">
         <f aca="false">E15</f>
         <v>0</v>
       </c>
-      <c r="G34" s="30"/>
-      <c r="H34" s="30"/>
+      <c r="G34" s="25"/>
+      <c r="H34" s="25"/>
       <c r="I34" s="4"/>
       <c r="J34" s="4"/>
       <c r="K34" s="4"/>
@@ -1815,11 +1800,11 @@
         <f aca="false">B34 &amp; " 5-Yr"</f>
         <v>PBV 5-Yr</v>
       </c>
-      <c r="C35" s="39"/>
-      <c r="D35" s="39"/>
-      <c r="E35" s="20"/>
-      <c r="G35" s="30"/>
-      <c r="H35" s="30"/>
+      <c r="C35" s="17"/>
+      <c r="D35" s="17"/>
+      <c r="E35" s="17"/>
+      <c r="G35" s="25"/>
+      <c r="H35" s="25"/>
       <c r="I35" s="4"/>
       <c r="J35" s="4"/>
       <c r="K35" s="4"/>
@@ -1835,24 +1820,24 @@
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="4"/>
-      <c r="B36" s="32" t="str">
+      <c r="B36" s="26" t="str">
         <f aca="false">"Valuacion " &amp; B35</f>
         <v>Valuacion PBV 5-Yr</v>
       </c>
-      <c r="C36" s="35" t="e">
+      <c r="C36" s="27" t="e">
         <f aca="false">(C$18*C35)/C34</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D36" s="35" t="e">
+      <c r="D36" s="27" t="e">
         <f aca="false">(D$18*D35)/D34</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E36" s="36" t="e">
+      <c r="E36" s="28" t="e">
         <f aca="false">(E$18*E35)/E34</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="G36" s="30"/>
-      <c r="H36" s="30"/>
+      <c r="G36" s="25"/>
+      <c r="H36" s="25"/>
       <c r="I36" s="4"/>
       <c r="J36" s="4"/>
       <c r="K36" s="4"/>
@@ -1868,13 +1853,13 @@
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="4"/>
-      <c r="B37" s="30"/>
-      <c r="C37" s="30"/>
-      <c r="D37" s="30"/>
-      <c r="E37" s="30"/>
-      <c r="F37" s="30"/>
-      <c r="G37" s="30"/>
-      <c r="H37" s="30"/>
+      <c r="B37" s="25"/>
+      <c r="C37" s="25"/>
+      <c r="D37" s="25"/>
+      <c r="E37" s="25"/>
+      <c r="F37" s="25"/>
+      <c r="G37" s="25"/>
+      <c r="H37" s="25"/>
       <c r="I37" s="4"/>
       <c r="J37" s="4"/>
       <c r="K37" s="4"/>
@@ -1891,21 +1876,21 @@
     <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="4"/>
       <c r="B38" s="8"/>
-      <c r="C38" s="40" t="n">
+      <c r="C38" s="31" t="n">
         <f aca="false">C2</f>
         <v>0</v>
       </c>
-      <c r="D38" s="40" t="n">
+      <c r="D38" s="31" t="n">
         <f aca="false">D2</f>
         <v>0</v>
       </c>
-      <c r="E38" s="40" t="n">
+      <c r="E38" s="31" t="n">
         <f aca="false">E2</f>
         <v>0</v>
       </c>
-      <c r="F38" s="30"/>
-      <c r="G38" s="30"/>
-      <c r="H38" s="30"/>
+      <c r="F38" s="25"/>
+      <c r="G38" s="25"/>
+      <c r="H38" s="25"/>
       <c r="I38" s="4"/>
       <c r="J38" s="4"/>
       <c r="K38" s="4"/>
@@ -1921,24 +1906,24 @@
     </row>
     <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="4"/>
-      <c r="B39" s="41" t="s">
+      <c r="B39" s="32" t="s">
         <v>22</v>
       </c>
-      <c r="C39" s="42" t="e">
+      <c r="C39" s="33" t="e">
         <f aca="false">AVERAGE(C27, C30, C33,C36)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D39" s="42" t="e">
+      <c r="D39" s="33" t="e">
         <f aca="false">AVERAGE(D27, D30, D33,D36)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E39" s="42" t="e">
+      <c r="E39" s="33" t="e">
         <f aca="false">AVERAGE(E27, E30, E33,E36)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="F39" s="30"/>
-      <c r="G39" s="30"/>
-      <c r="H39" s="30"/>
+      <c r="F39" s="25"/>
+      <c r="G39" s="25"/>
+      <c r="H39" s="25"/>
       <c r="I39" s="4"/>
       <c r="J39" s="4"/>
       <c r="K39" s="4"/>
@@ -1957,21 +1942,21 @@
       <c r="B40" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="C40" s="43" t="e">
+      <c r="C40" s="34" t="e">
         <f aca="false">AVERAGE(C19:C22)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D40" s="43" t="e">
+      <c r="D40" s="34" t="e">
         <f aca="false">AVERAGE(D19:D22)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E40" s="43" t="e">
+      <c r="E40" s="34" t="e">
         <f aca="false">AVERAGE(E19:E22)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="F40" s="30"/>
-      <c r="G40" s="30"/>
-      <c r="H40" s="30"/>
+      <c r="F40" s="25"/>
+      <c r="G40" s="25"/>
+      <c r="H40" s="25"/>
       <c r="I40" s="4"/>
       <c r="J40" s="4"/>
       <c r="K40" s="4"/>
@@ -1987,24 +1972,24 @@
     </row>
     <row r="41" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="4"/>
-      <c r="B41" s="44" t="s">
+      <c r="B41" s="35" t="s">
         <v>24</v>
       </c>
-      <c r="C41" s="45" t="e">
+      <c r="C41" s="36" t="e">
         <f aca="false">AVERAGE(C39:C40)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D41" s="45" t="e">
+      <c r="D41" s="36" t="e">
         <f aca="false">AVERAGE(D39:D40)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E41" s="45" t="e">
+      <c r="E41" s="36" t="e">
         <f aca="false">AVERAGE(E39:E40)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="F41" s="30"/>
-      <c r="G41" s="30"/>
-      <c r="H41" s="30"/>
+      <c r="F41" s="25"/>
+      <c r="G41" s="25"/>
+      <c r="H41" s="25"/>
       <c r="I41" s="4"/>
       <c r="J41" s="4"/>
       <c r="K41" s="4"/>
@@ -2021,12 +2006,12 @@
     <row r="42" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="4"/>
       <c r="B42" s="8"/>
-      <c r="C42" s="15"/>
-      <c r="D42" s="15"/>
-      <c r="E42" s="15"/>
-      <c r="F42" s="30"/>
-      <c r="G42" s="30"/>
-      <c r="H42" s="30"/>
+      <c r="C42" s="37"/>
+      <c r="D42" s="37"/>
+      <c r="E42" s="37"/>
+      <c r="F42" s="25"/>
+      <c r="G42" s="25"/>
+      <c r="H42" s="25"/>
       <c r="I42" s="4"/>
       <c r="J42" s="4"/>
       <c r="K42" s="4"/>
@@ -2042,24 +2027,24 @@
     </row>
     <row r="43" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="4"/>
-      <c r="B43" s="46" t="s">
+      <c r="B43" s="38" t="s">
         <v>25</v>
       </c>
-      <c r="C43" s="47" t="e">
+      <c r="C43" s="39" t="e">
         <f aca="false">(C$18-C41)/C$18</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D43" s="47" t="e">
+      <c r="D43" s="39" t="e">
         <f aca="false">(D$18-D41)/D$18</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E43" s="47" t="e">
+      <c r="E43" s="39" t="e">
         <f aca="false">(E$18-E41)/E$18</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="F43" s="30"/>
-      <c r="G43" s="30"/>
-      <c r="H43" s="30"/>
+      <c r="F43" s="25"/>
+      <c r="G43" s="25"/>
+      <c r="H43" s="25"/>
       <c r="I43" s="4"/>
       <c r="J43" s="4"/>
       <c r="K43" s="4"/>
@@ -2075,25 +2060,25 @@
     </row>
     <row r="44" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="4"/>
-      <c r="B44" s="46" t="str">
+      <c r="B44" s="38" t="str">
         <f aca="false">"Diff " &amp; B26 &amp; " %"</f>
         <v>Diff PER 5-Yr %</v>
       </c>
-      <c r="C44" s="47" t="e">
+      <c r="C44" s="39" t="e">
         <f aca="false">(C$18-C27)/C$18</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D44" s="47" t="e">
+      <c r="D44" s="39" t="e">
         <f aca="false">(D$18-D27)/D$18</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E44" s="47" t="e">
+      <c r="E44" s="39" t="e">
         <f aca="false">(E$18-E27)/E$18</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="F44" s="30"/>
-      <c r="G44" s="30"/>
-      <c r="H44" s="30"/>
+      <c r="F44" s="25"/>
+      <c r="G44" s="25"/>
+      <c r="H44" s="25"/>
       <c r="I44" s="4"/>
       <c r="J44" s="4"/>
       <c r="K44" s="4"/>
@@ -2109,19 +2094,19 @@
     </row>
     <row r="45" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="4"/>
-      <c r="B45" s="46" t="str">
+      <c r="B45" s="38" t="str">
         <f aca="false">"Diff " &amp; B29 &amp; " %"</f>
         <v>Diff PCF 5-Yr %</v>
       </c>
-      <c r="C45" s="47" t="e">
+      <c r="C45" s="39" t="e">
         <f aca="false">(C$18-C30)/C$18</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D45" s="47" t="e">
+      <c r="D45" s="39" t="e">
         <f aca="false">(D$18-D30)/D$18</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E45" s="47" t="e">
+      <c r="E45" s="39" t="e">
         <f aca="false">(E$18-E30)/E$18</f>
         <v>#DIV/0!</v>
       </c>
@@ -2143,19 +2128,19 @@
     </row>
     <row r="46" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="4"/>
-      <c r="B46" s="46" t="str">
+      <c r="B46" s="38" t="str">
         <f aca="false">"Diff " &amp; B32 &amp; " %"</f>
         <v>Diff PS 5-Yr %</v>
       </c>
-      <c r="C46" s="47" t="e">
+      <c r="C46" s="39" t="e">
         <f aca="false">(C$18-C33)/C$18</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D46" s="47" t="e">
+      <c r="D46" s="39" t="e">
         <f aca="false">(D$18-D33)/D$18</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E46" s="47" t="e">
+      <c r="E46" s="39" t="e">
         <f aca="false">(E$18-E33)/E$18</f>
         <v>#DIV/0!</v>
       </c>
@@ -2177,19 +2162,19 @@
     </row>
     <row r="47" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="4"/>
-      <c r="B47" s="46" t="str">
+      <c r="B47" s="38" t="str">
         <f aca="false">"Diff " &amp; B35 &amp; " %"</f>
         <v>Diff PBV 5-Yr %</v>
       </c>
-      <c r="C47" s="47" t="e">
+      <c r="C47" s="39" t="e">
         <f aca="false">(C$18-C36)/C$18</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D47" s="47" t="e">
+      <c r="D47" s="39" t="e">
         <f aca="false">(D$18-D36)/D$18</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E47" s="47" t="e">
+      <c r="E47" s="39" t="e">
         <f aca="false">(E$18-E36)/E$18</f>
         <v>#DIV/0!</v>
       </c>
@@ -2232,20 +2217,22 @@
       <c r="T48" s="4"/>
     </row>
     <row r="49" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B49" s="4"/>
-      <c r="C49" s="4"/>
-      <c r="D49" s="4"/>
-      <c r="E49" s="4"/>
-      <c r="F49" s="4"/>
-      <c r="G49" s="4"/>
-      <c r="H49" s="4"/>
-      <c r="I49" s="4"/>
-      <c r="J49" s="4"/>
-      <c r="K49" s="4"/>
-      <c r="L49" s="4"/>
-      <c r="M49" s="4"/>
-      <c r="N49" s="4"/>
-      <c r="O49" s="4"/>
+      <c r="B49" s="40" t="s">
+        <v>26</v>
+      </c>
+      <c r="C49" s="40"/>
+      <c r="D49" s="40"/>
+      <c r="E49" s="40"/>
+      <c r="F49" s="40"/>
+      <c r="G49" s="40"/>
+      <c r="H49" s="40"/>
+      <c r="I49" s="40"/>
+      <c r="J49" s="40"/>
+      <c r="K49" s="40"/>
+      <c r="L49" s="40"/>
+      <c r="M49" s="40"/>
+      <c r="N49" s="40"/>
+      <c r="O49" s="40"/>
       <c r="P49" s="4"/>
       <c r="Q49" s="4"/>
       <c r="R49" s="4"/>
@@ -2253,20 +2240,20 @@
       <c r="T49" s="4"/>
     </row>
     <row r="50" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B50" s="4"/>
-      <c r="C50" s="4"/>
-      <c r="D50" s="4"/>
-      <c r="E50" s="4"/>
-      <c r="F50" s="4"/>
-      <c r="G50" s="4"/>
-      <c r="H50" s="4"/>
-      <c r="I50" s="4"/>
-      <c r="J50" s="4"/>
-      <c r="K50" s="4"/>
-      <c r="L50" s="4"/>
-      <c r="M50" s="4"/>
-      <c r="N50" s="4"/>
-      <c r="O50" s="4"/>
+      <c r="B50" s="40"/>
+      <c r="C50" s="40"/>
+      <c r="D50" s="40"/>
+      <c r="E50" s="40"/>
+      <c r="F50" s="40"/>
+      <c r="G50" s="40"/>
+      <c r="H50" s="40"/>
+      <c r="I50" s="40"/>
+      <c r="J50" s="40"/>
+      <c r="K50" s="40"/>
+      <c r="L50" s="40"/>
+      <c r="M50" s="40"/>
+      <c r="N50" s="40"/>
+      <c r="O50" s="40"/>
       <c r="P50" s="4"/>
       <c r="Q50" s="4"/>
       <c r="R50" s="4"/>
@@ -2274,20 +2261,20 @@
       <c r="T50" s="4"/>
     </row>
     <row r="51" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B51" s="4"/>
-      <c r="C51" s="4"/>
-      <c r="D51" s="4"/>
-      <c r="E51" s="4"/>
-      <c r="F51" s="4"/>
-      <c r="G51" s="4"/>
-      <c r="H51" s="4"/>
-      <c r="I51" s="4"/>
-      <c r="J51" s="4"/>
-      <c r="K51" s="4"/>
-      <c r="L51" s="4"/>
-      <c r="M51" s="4"/>
-      <c r="N51" s="4"/>
-      <c r="O51" s="4"/>
+      <c r="B51" s="40"/>
+      <c r="C51" s="40"/>
+      <c r="D51" s="40"/>
+      <c r="E51" s="40"/>
+      <c r="F51" s="40"/>
+      <c r="G51" s="40"/>
+      <c r="H51" s="40"/>
+      <c r="I51" s="40"/>
+      <c r="J51" s="40"/>
+      <c r="K51" s="40"/>
+      <c r="L51" s="40"/>
+      <c r="M51" s="40"/>
+      <c r="N51" s="40"/>
+      <c r="O51" s="40"/>
       <c r="P51" s="4"/>
       <c r="Q51" s="4"/>
       <c r="R51" s="4"/>
@@ -2295,20 +2282,20 @@
       <c r="T51" s="4"/>
     </row>
     <row r="52" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B52" s="4"/>
-      <c r="C52" s="4"/>
-      <c r="D52" s="4"/>
-      <c r="E52" s="4"/>
-      <c r="F52" s="4"/>
-      <c r="G52" s="4"/>
-      <c r="H52" s="4"/>
-      <c r="I52" s="4"/>
-      <c r="J52" s="4"/>
-      <c r="K52" s="4"/>
-      <c r="L52" s="4"/>
-      <c r="M52" s="4"/>
-      <c r="N52" s="4"/>
-      <c r="O52" s="4"/>
+      <c r="B52" s="40"/>
+      <c r="C52" s="40"/>
+      <c r="D52" s="40"/>
+      <c r="E52" s="40"/>
+      <c r="F52" s="40"/>
+      <c r="G52" s="40"/>
+      <c r="H52" s="40"/>
+      <c r="I52" s="40"/>
+      <c r="J52" s="40"/>
+      <c r="K52" s="40"/>
+      <c r="L52" s="40"/>
+      <c r="M52" s="40"/>
+      <c r="N52" s="40"/>
+      <c r="O52" s="40"/>
       <c r="P52" s="4"/>
       <c r="Q52" s="4"/>
       <c r="R52" s="4"/>
@@ -2316,20 +2303,20 @@
       <c r="T52" s="4"/>
     </row>
     <row r="53" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B53" s="4"/>
-      <c r="C53" s="4"/>
-      <c r="D53" s="4"/>
-      <c r="E53" s="4"/>
-      <c r="F53" s="4"/>
-      <c r="G53" s="4"/>
-      <c r="H53" s="4"/>
-      <c r="I53" s="4"/>
-      <c r="J53" s="4"/>
-      <c r="K53" s="4"/>
-      <c r="L53" s="4"/>
-      <c r="M53" s="4"/>
-      <c r="N53" s="4"/>
-      <c r="O53" s="4"/>
+      <c r="B53" s="40"/>
+      <c r="C53" s="40"/>
+      <c r="D53" s="40"/>
+      <c r="E53" s="40"/>
+      <c r="F53" s="40"/>
+      <c r="G53" s="40"/>
+      <c r="H53" s="40"/>
+      <c r="I53" s="40"/>
+      <c r="J53" s="40"/>
+      <c r="K53" s="40"/>
+      <c r="L53" s="40"/>
+      <c r="M53" s="40"/>
+      <c r="N53" s="40"/>
+      <c r="O53" s="40"/>
       <c r="P53" s="4"/>
       <c r="Q53" s="4"/>
       <c r="R53" s="4"/>
@@ -2337,20 +2324,20 @@
       <c r="T53" s="4"/>
     </row>
     <row r="54" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B54" s="4"/>
-      <c r="C54" s="4"/>
-      <c r="D54" s="4"/>
-      <c r="E54" s="4"/>
-      <c r="F54" s="4"/>
-      <c r="G54" s="4"/>
-      <c r="H54" s="4"/>
-      <c r="I54" s="4"/>
-      <c r="J54" s="4"/>
-      <c r="K54" s="4"/>
-      <c r="L54" s="4"/>
-      <c r="M54" s="4"/>
-      <c r="N54" s="4"/>
-      <c r="O54" s="4"/>
+      <c r="B54" s="40"/>
+      <c r="C54" s="40"/>
+      <c r="D54" s="40"/>
+      <c r="E54" s="40"/>
+      <c r="F54" s="40"/>
+      <c r="G54" s="40"/>
+      <c r="H54" s="40"/>
+      <c r="I54" s="40"/>
+      <c r="J54" s="40"/>
+      <c r="K54" s="40"/>
+      <c r="L54" s="40"/>
+      <c r="M54" s="40"/>
+      <c r="N54" s="40"/>
+      <c r="O54" s="40"/>
       <c r="P54" s="4"/>
       <c r="Q54" s="4"/>
       <c r="R54" s="4"/>
@@ -2358,20 +2345,20 @@
       <c r="T54" s="4"/>
     </row>
     <row r="55" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B55" s="4"/>
-      <c r="C55" s="4"/>
-      <c r="D55" s="4"/>
-      <c r="E55" s="4"/>
-      <c r="F55" s="4"/>
-      <c r="G55" s="4"/>
-      <c r="H55" s="4"/>
-      <c r="I55" s="4"/>
-      <c r="J55" s="4"/>
-      <c r="K55" s="4"/>
-      <c r="L55" s="4"/>
-      <c r="M55" s="4"/>
-      <c r="N55" s="4"/>
-      <c r="O55" s="4"/>
+      <c r="B55" s="40"/>
+      <c r="C55" s="40"/>
+      <c r="D55" s="40"/>
+      <c r="E55" s="40"/>
+      <c r="F55" s="40"/>
+      <c r="G55" s="40"/>
+      <c r="H55" s="40"/>
+      <c r="I55" s="40"/>
+      <c r="J55" s="40"/>
+      <c r="K55" s="40"/>
+      <c r="L55" s="40"/>
+      <c r="M55" s="40"/>
+      <c r="N55" s="40"/>
+      <c r="O55" s="40"/>
       <c r="P55" s="4"/>
       <c r="Q55" s="4"/>
       <c r="R55" s="4"/>
@@ -2379,20 +2366,20 @@
       <c r="T55" s="4"/>
     </row>
     <row r="56" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B56" s="4"/>
-      <c r="C56" s="4"/>
-      <c r="D56" s="4"/>
-      <c r="E56" s="4"/>
-      <c r="F56" s="4"/>
-      <c r="G56" s="4"/>
-      <c r="H56" s="4"/>
-      <c r="I56" s="4"/>
-      <c r="J56" s="4"/>
-      <c r="K56" s="4"/>
-      <c r="L56" s="4"/>
-      <c r="M56" s="4"/>
-      <c r="N56" s="4"/>
-      <c r="O56" s="4"/>
+      <c r="B56" s="40"/>
+      <c r="C56" s="40"/>
+      <c r="D56" s="40"/>
+      <c r="E56" s="40"/>
+      <c r="F56" s="40"/>
+      <c r="G56" s="40"/>
+      <c r="H56" s="40"/>
+      <c r="I56" s="40"/>
+      <c r="J56" s="40"/>
+      <c r="K56" s="40"/>
+      <c r="L56" s="40"/>
+      <c r="M56" s="40"/>
+      <c r="N56" s="40"/>
+      <c r="O56" s="40"/>
       <c r="P56" s="4"/>
       <c r="Q56" s="4"/>
       <c r="R56" s="4"/>
@@ -2400,20 +2387,20 @@
       <c r="T56" s="4"/>
     </row>
     <row r="57" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B57" s="4"/>
-      <c r="C57" s="4"/>
-      <c r="D57" s="4"/>
-      <c r="E57" s="4"/>
-      <c r="F57" s="4"/>
-      <c r="G57" s="4"/>
-      <c r="H57" s="4"/>
-      <c r="I57" s="4"/>
-      <c r="J57" s="4"/>
-      <c r="K57" s="4"/>
-      <c r="L57" s="4"/>
-      <c r="M57" s="4"/>
-      <c r="N57" s="4"/>
-      <c r="O57" s="4"/>
+      <c r="B57" s="40"/>
+      <c r="C57" s="40"/>
+      <c r="D57" s="40"/>
+      <c r="E57" s="40"/>
+      <c r="F57" s="40"/>
+      <c r="G57" s="40"/>
+      <c r="H57" s="40"/>
+      <c r="I57" s="40"/>
+      <c r="J57" s="40"/>
+      <c r="K57" s="40"/>
+      <c r="L57" s="40"/>
+      <c r="M57" s="40"/>
+      <c r="N57" s="40"/>
+      <c r="O57" s="40"/>
       <c r="P57" s="4"/>
       <c r="Q57" s="4"/>
       <c r="R57" s="4"/>
@@ -2421,20 +2408,20 @@
       <c r="T57" s="4"/>
     </row>
     <row r="58" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B58" s="4"/>
-      <c r="C58" s="4"/>
-      <c r="D58" s="4"/>
-      <c r="E58" s="4"/>
-      <c r="F58" s="4"/>
-      <c r="G58" s="4"/>
-      <c r="H58" s="4"/>
-      <c r="I58" s="4"/>
-      <c r="J58" s="4"/>
-      <c r="K58" s="4"/>
-      <c r="L58" s="4"/>
-      <c r="M58" s="4"/>
-      <c r="N58" s="4"/>
-      <c r="O58" s="4"/>
+      <c r="B58" s="40"/>
+      <c r="C58" s="40"/>
+      <c r="D58" s="40"/>
+      <c r="E58" s="40"/>
+      <c r="F58" s="40"/>
+      <c r="G58" s="40"/>
+      <c r="H58" s="40"/>
+      <c r="I58" s="40"/>
+      <c r="J58" s="40"/>
+      <c r="K58" s="40"/>
+      <c r="L58" s="40"/>
+      <c r="M58" s="40"/>
+      <c r="N58" s="40"/>
+      <c r="O58" s="40"/>
       <c r="P58" s="4"/>
       <c r="Q58" s="4"/>
       <c r="R58" s="4"/>
@@ -2442,20 +2429,20 @@
       <c r="T58" s="4"/>
     </row>
     <row r="59" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B59" s="4"/>
-      <c r="C59" s="4"/>
-      <c r="D59" s="4"/>
-      <c r="E59" s="4"/>
-      <c r="F59" s="4"/>
-      <c r="G59" s="4"/>
-      <c r="H59" s="4"/>
-      <c r="I59" s="4"/>
-      <c r="J59" s="4"/>
-      <c r="K59" s="4"/>
-      <c r="L59" s="4"/>
-      <c r="M59" s="4"/>
-      <c r="N59" s="4"/>
-      <c r="O59" s="4"/>
+      <c r="B59" s="40"/>
+      <c r="C59" s="40"/>
+      <c r="D59" s="40"/>
+      <c r="E59" s="40"/>
+      <c r="F59" s="40"/>
+      <c r="G59" s="40"/>
+      <c r="H59" s="40"/>
+      <c r="I59" s="40"/>
+      <c r="J59" s="40"/>
+      <c r="K59" s="40"/>
+      <c r="L59" s="40"/>
+      <c r="M59" s="40"/>
+      <c r="N59" s="40"/>
+      <c r="O59" s="40"/>
       <c r="P59" s="4"/>
       <c r="Q59" s="4"/>
       <c r="R59" s="4"/>
@@ -2463,20 +2450,20 @@
       <c r="T59" s="4"/>
     </row>
     <row r="60" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B60" s="4"/>
-      <c r="C60" s="4"/>
-      <c r="D60" s="4"/>
-      <c r="E60" s="4"/>
-      <c r="F60" s="4"/>
-      <c r="G60" s="4"/>
-      <c r="H60" s="4"/>
-      <c r="I60" s="4"/>
-      <c r="J60" s="4"/>
-      <c r="K60" s="4"/>
-      <c r="L60" s="4"/>
-      <c r="M60" s="4"/>
-      <c r="N60" s="4"/>
-      <c r="O60" s="4"/>
+      <c r="B60" s="40"/>
+      <c r="C60" s="40"/>
+      <c r="D60" s="40"/>
+      <c r="E60" s="40"/>
+      <c r="F60" s="40"/>
+      <c r="G60" s="40"/>
+      <c r="H60" s="40"/>
+      <c r="I60" s="40"/>
+      <c r="J60" s="40"/>
+      <c r="K60" s="40"/>
+      <c r="L60" s="40"/>
+      <c r="M60" s="40"/>
+      <c r="N60" s="40"/>
+      <c r="O60" s="40"/>
       <c r="P60" s="4"/>
       <c r="Q60" s="4"/>
       <c r="R60" s="4"/>
@@ -2484,20 +2471,20 @@
       <c r="T60" s="4"/>
     </row>
     <row r="61" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B61" s="4"/>
-      <c r="C61" s="4"/>
-      <c r="D61" s="4"/>
-      <c r="E61" s="4"/>
-      <c r="F61" s="4"/>
-      <c r="G61" s="4"/>
-      <c r="H61" s="4"/>
-      <c r="I61" s="4"/>
-      <c r="J61" s="4"/>
-      <c r="K61" s="4"/>
-      <c r="L61" s="4"/>
-      <c r="M61" s="4"/>
-      <c r="N61" s="4"/>
-      <c r="O61" s="4"/>
+      <c r="B61" s="40"/>
+      <c r="C61" s="40"/>
+      <c r="D61" s="40"/>
+      <c r="E61" s="40"/>
+      <c r="F61" s="40"/>
+      <c r="G61" s="40"/>
+      <c r="H61" s="40"/>
+      <c r="I61" s="40"/>
+      <c r="J61" s="40"/>
+      <c r="K61" s="40"/>
+      <c r="L61" s="40"/>
+      <c r="M61" s="40"/>
+      <c r="N61" s="40"/>
+      <c r="O61" s="40"/>
       <c r="P61" s="4"/>
       <c r="Q61" s="4"/>
       <c r="R61" s="4"/>
@@ -2505,20 +2492,20 @@
       <c r="T61" s="4"/>
     </row>
     <row r="62" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B62" s="4"/>
-      <c r="C62" s="4"/>
-      <c r="D62" s="4"/>
-      <c r="E62" s="4"/>
-      <c r="F62" s="4"/>
-      <c r="G62" s="4"/>
-      <c r="H62" s="4"/>
-      <c r="I62" s="4"/>
-      <c r="J62" s="4"/>
-      <c r="K62" s="4"/>
-      <c r="L62" s="4"/>
-      <c r="M62" s="4"/>
-      <c r="N62" s="4"/>
-      <c r="O62" s="4"/>
+      <c r="B62" s="40"/>
+      <c r="C62" s="40"/>
+      <c r="D62" s="40"/>
+      <c r="E62" s="40"/>
+      <c r="F62" s="40"/>
+      <c r="G62" s="40"/>
+      <c r="H62" s="40"/>
+      <c r="I62" s="40"/>
+      <c r="J62" s="40"/>
+      <c r="K62" s="40"/>
+      <c r="L62" s="40"/>
+      <c r="M62" s="40"/>
+      <c r="N62" s="40"/>
+      <c r="O62" s="40"/>
       <c r="P62" s="4"/>
       <c r="Q62" s="4"/>
       <c r="R62" s="4"/>
@@ -2526,20 +2513,20 @@
       <c r="T62" s="4"/>
     </row>
     <row r="63" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B63" s="4"/>
-      <c r="C63" s="4"/>
-      <c r="D63" s="4"/>
-      <c r="E63" s="4"/>
-      <c r="F63" s="4"/>
-      <c r="G63" s="4"/>
-      <c r="H63" s="4"/>
-      <c r="I63" s="4"/>
-      <c r="J63" s="4"/>
-      <c r="K63" s="4"/>
-      <c r="L63" s="4"/>
-      <c r="M63" s="4"/>
-      <c r="N63" s="4"/>
-      <c r="O63" s="4"/>
+      <c r="B63" s="40"/>
+      <c r="C63" s="40"/>
+      <c r="D63" s="40"/>
+      <c r="E63" s="40"/>
+      <c r="F63" s="40"/>
+      <c r="G63" s="40"/>
+      <c r="H63" s="40"/>
+      <c r="I63" s="40"/>
+      <c r="J63" s="40"/>
+      <c r="K63" s="40"/>
+      <c r="L63" s="40"/>
+      <c r="M63" s="40"/>
+      <c r="N63" s="40"/>
+      <c r="O63" s="40"/>
       <c r="P63" s="4"/>
       <c r="Q63" s="4"/>
       <c r="R63" s="4"/>
@@ -2547,20 +2534,20 @@
       <c r="T63" s="4"/>
     </row>
     <row r="64" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B64" s="4"/>
-      <c r="C64" s="4"/>
-      <c r="D64" s="4"/>
-      <c r="E64" s="4"/>
-      <c r="F64" s="4"/>
-      <c r="G64" s="4"/>
-      <c r="H64" s="4"/>
-      <c r="I64" s="4"/>
-      <c r="J64" s="4"/>
-      <c r="K64" s="4"/>
-      <c r="L64" s="4"/>
-      <c r="M64" s="4"/>
-      <c r="N64" s="4"/>
-      <c r="O64" s="4"/>
+      <c r="B64" s="40"/>
+      <c r="C64" s="40"/>
+      <c r="D64" s="40"/>
+      <c r="E64" s="40"/>
+      <c r="F64" s="40"/>
+      <c r="G64" s="40"/>
+      <c r="H64" s="40"/>
+      <c r="I64" s="40"/>
+      <c r="J64" s="40"/>
+      <c r="K64" s="40"/>
+      <c r="L64" s="40"/>
+      <c r="M64" s="40"/>
+      <c r="N64" s="40"/>
+      <c r="O64" s="40"/>
       <c r="P64" s="4"/>
       <c r="Q64" s="4"/>
       <c r="R64" s="4"/>
@@ -2568,20 +2555,20 @@
       <c r="T64" s="4"/>
     </row>
     <row r="65" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B65" s="4"/>
-      <c r="C65" s="4"/>
-      <c r="D65" s="4"/>
-      <c r="E65" s="4"/>
-      <c r="F65" s="4"/>
-      <c r="G65" s="4"/>
-      <c r="H65" s="4"/>
-      <c r="I65" s="4"/>
-      <c r="J65" s="4"/>
-      <c r="K65" s="4"/>
-      <c r="L65" s="4"/>
-      <c r="M65" s="4"/>
-      <c r="N65" s="4"/>
-      <c r="O65" s="4"/>
+      <c r="B65" s="40"/>
+      <c r="C65" s="40"/>
+      <c r="D65" s="40"/>
+      <c r="E65" s="40"/>
+      <c r="F65" s="40"/>
+      <c r="G65" s="40"/>
+      <c r="H65" s="40"/>
+      <c r="I65" s="40"/>
+      <c r="J65" s="40"/>
+      <c r="K65" s="40"/>
+      <c r="L65" s="40"/>
+      <c r="M65" s="40"/>
+      <c r="N65" s="40"/>
+      <c r="O65" s="40"/>
       <c r="P65" s="4"/>
       <c r="Q65" s="4"/>
       <c r="R65" s="4"/>
@@ -2589,20 +2576,20 @@
       <c r="T65" s="4"/>
     </row>
     <row r="66" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B66" s="4"/>
-      <c r="C66" s="4"/>
-      <c r="D66" s="4"/>
-      <c r="E66" s="4"/>
-      <c r="F66" s="4"/>
-      <c r="G66" s="4"/>
-      <c r="H66" s="4"/>
-      <c r="I66" s="4"/>
-      <c r="J66" s="4"/>
-      <c r="K66" s="4"/>
-      <c r="L66" s="4"/>
-      <c r="M66" s="4"/>
-      <c r="N66" s="4"/>
-      <c r="O66" s="4"/>
+      <c r="B66" s="40"/>
+      <c r="C66" s="40"/>
+      <c r="D66" s="40"/>
+      <c r="E66" s="40"/>
+      <c r="F66" s="40"/>
+      <c r="G66" s="40"/>
+      <c r="H66" s="40"/>
+      <c r="I66" s="40"/>
+      <c r="J66" s="40"/>
+      <c r="K66" s="40"/>
+      <c r="L66" s="40"/>
+      <c r="M66" s="40"/>
+      <c r="N66" s="40"/>
+      <c r="O66" s="40"/>
       <c r="P66" s="4"/>
       <c r="Q66" s="4"/>
       <c r="R66" s="4"/>
@@ -2610,20 +2597,20 @@
       <c r="T66" s="4"/>
     </row>
     <row r="67" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B67" s="4"/>
-      <c r="C67" s="4"/>
-      <c r="D67" s="4"/>
-      <c r="E67" s="4"/>
-      <c r="F67" s="4"/>
-      <c r="G67" s="4"/>
-      <c r="H67" s="4"/>
-      <c r="I67" s="4"/>
-      <c r="J67" s="4"/>
-      <c r="K67" s="4"/>
-      <c r="L67" s="4"/>
-      <c r="M67" s="4"/>
-      <c r="N67" s="4"/>
-      <c r="O67" s="4"/>
+      <c r="B67" s="40"/>
+      <c r="C67" s="40"/>
+      <c r="D67" s="40"/>
+      <c r="E67" s="40"/>
+      <c r="F67" s="40"/>
+      <c r="G67" s="40"/>
+      <c r="H67" s="40"/>
+      <c r="I67" s="40"/>
+      <c r="J67" s="40"/>
+      <c r="K67" s="40"/>
+      <c r="L67" s="40"/>
+      <c r="M67" s="40"/>
+      <c r="N67" s="40"/>
+      <c r="O67" s="40"/>
       <c r="P67" s="4"/>
       <c r="Q67" s="4"/>
       <c r="R67" s="4"/>
@@ -2631,20 +2618,20 @@
       <c r="T67" s="4"/>
     </row>
     <row r="68" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B68" s="4"/>
-      <c r="C68" s="4"/>
-      <c r="D68" s="4"/>
-      <c r="E68" s="4"/>
-      <c r="F68" s="4"/>
-      <c r="G68" s="4"/>
-      <c r="H68" s="4"/>
-      <c r="I68" s="4"/>
-      <c r="J68" s="4"/>
-      <c r="K68" s="4"/>
-      <c r="L68" s="4"/>
-      <c r="M68" s="4"/>
-      <c r="N68" s="4"/>
-      <c r="O68" s="4"/>
+      <c r="B68" s="40"/>
+      <c r="C68" s="40"/>
+      <c r="D68" s="40"/>
+      <c r="E68" s="40"/>
+      <c r="F68" s="40"/>
+      <c r="G68" s="40"/>
+      <c r="H68" s="40"/>
+      <c r="I68" s="40"/>
+      <c r="J68" s="40"/>
+      <c r="K68" s="40"/>
+      <c r="L68" s="40"/>
+      <c r="M68" s="40"/>
+      <c r="N68" s="40"/>
+      <c r="O68" s="40"/>
       <c r="P68" s="4"/>
       <c r="Q68" s="4"/>
       <c r="R68" s="4"/>
@@ -2652,20 +2639,20 @@
       <c r="T68" s="4"/>
     </row>
     <row r="69" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B69" s="4"/>
-      <c r="C69" s="4"/>
-      <c r="D69" s="4"/>
-      <c r="E69" s="4"/>
-      <c r="F69" s="4"/>
-      <c r="G69" s="4"/>
-      <c r="H69" s="4"/>
-      <c r="I69" s="4"/>
-      <c r="J69" s="4"/>
-      <c r="K69" s="4"/>
-      <c r="L69" s="4"/>
-      <c r="M69" s="4"/>
-      <c r="N69" s="4"/>
-      <c r="O69" s="4"/>
+      <c r="B69" s="40"/>
+      <c r="C69" s="40"/>
+      <c r="D69" s="40"/>
+      <c r="E69" s="40"/>
+      <c r="F69" s="40"/>
+      <c r="G69" s="40"/>
+      <c r="H69" s="40"/>
+      <c r="I69" s="40"/>
+      <c r="J69" s="40"/>
+      <c r="K69" s="40"/>
+      <c r="L69" s="40"/>
+      <c r="M69" s="40"/>
+      <c r="N69" s="40"/>
+      <c r="O69" s="40"/>
       <c r="P69" s="4"/>
       <c r="Q69" s="4"/>
       <c r="R69" s="4"/>
@@ -2673,20 +2660,20 @@
       <c r="T69" s="4"/>
     </row>
     <row r="70" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B70" s="4"/>
-      <c r="C70" s="4"/>
-      <c r="D70" s="4"/>
-      <c r="E70" s="4"/>
-      <c r="F70" s="4"/>
-      <c r="G70" s="4"/>
-      <c r="H70" s="4"/>
-      <c r="I70" s="4"/>
-      <c r="J70" s="4"/>
-      <c r="K70" s="4"/>
-      <c r="L70" s="4"/>
-      <c r="M70" s="4"/>
-      <c r="N70" s="4"/>
-      <c r="O70" s="4"/>
+      <c r="B70" s="40"/>
+      <c r="C70" s="40"/>
+      <c r="D70" s="40"/>
+      <c r="E70" s="40"/>
+      <c r="F70" s="40"/>
+      <c r="G70" s="40"/>
+      <c r="H70" s="40"/>
+      <c r="I70" s="40"/>
+      <c r="J70" s="40"/>
+      <c r="K70" s="40"/>
+      <c r="L70" s="40"/>
+      <c r="M70" s="40"/>
+      <c r="N70" s="40"/>
+      <c r="O70" s="40"/>
       <c r="P70" s="4"/>
       <c r="Q70" s="4"/>
       <c r="R70" s="4"/>
@@ -2694,20 +2681,20 @@
       <c r="T70" s="4"/>
     </row>
     <row r="71" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B71" s="4"/>
-      <c r="C71" s="4"/>
-      <c r="D71" s="4"/>
-      <c r="E71" s="4"/>
-      <c r="F71" s="4"/>
-      <c r="G71" s="4"/>
-      <c r="H71" s="4"/>
-      <c r="I71" s="4"/>
-      <c r="J71" s="4"/>
-      <c r="K71" s="4"/>
-      <c r="L71" s="4"/>
-      <c r="M71" s="4"/>
-      <c r="N71" s="4"/>
-      <c r="O71" s="4"/>
+      <c r="B71" s="40"/>
+      <c r="C71" s="40"/>
+      <c r="D71" s="40"/>
+      <c r="E71" s="40"/>
+      <c r="F71" s="40"/>
+      <c r="G71" s="40"/>
+      <c r="H71" s="40"/>
+      <c r="I71" s="40"/>
+      <c r="J71" s="40"/>
+      <c r="K71" s="40"/>
+      <c r="L71" s="40"/>
+      <c r="M71" s="40"/>
+      <c r="N71" s="40"/>
+      <c r="O71" s="40"/>
       <c r="P71" s="4"/>
       <c r="Q71" s="4"/>
       <c r="R71" s="4"/>
@@ -2715,20 +2702,20 @@
       <c r="T71" s="4"/>
     </row>
     <row r="72" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B72" s="4"/>
-      <c r="C72" s="4"/>
-      <c r="D72" s="4"/>
-      <c r="E72" s="4"/>
-      <c r="F72" s="4"/>
-      <c r="G72" s="4"/>
-      <c r="H72" s="4"/>
-      <c r="I72" s="4"/>
-      <c r="J72" s="4"/>
-      <c r="K72" s="4"/>
-      <c r="L72" s="4"/>
-      <c r="M72" s="4"/>
-      <c r="N72" s="4"/>
-      <c r="O72" s="4"/>
+      <c r="B72" s="40"/>
+      <c r="C72" s="40"/>
+      <c r="D72" s="40"/>
+      <c r="E72" s="40"/>
+      <c r="F72" s="40"/>
+      <c r="G72" s="40"/>
+      <c r="H72" s="40"/>
+      <c r="I72" s="40"/>
+      <c r="J72" s="40"/>
+      <c r="K72" s="40"/>
+      <c r="L72" s="40"/>
+      <c r="M72" s="40"/>
+      <c r="N72" s="40"/>
+      <c r="O72" s="40"/>
       <c r="P72" s="4"/>
       <c r="Q72" s="4"/>
       <c r="R72" s="4"/>

</xml_diff>